<commit_message>
updated after match 6
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9856C168-1D0D-4752-A231-8C09A0C8D7B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D65B4BB4-F8EC-4022-9401-6D18BB2BE06C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
@@ -1042,16 +1042,16 @@
     </row>
     <row r="3" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>120</v>
+        <v>66</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C3" s="1">
         <v>0</v>
       </c>
       <c r="D3" s="1">
-        <v>166</v>
+        <v>52</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>1</v>
@@ -1081,37 +1081,37 @@
         <v>0</v>
       </c>
       <c r="N3" s="1">
-        <v>71</v>
+        <v>159</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="R3" s="1">
         <v>0</v>
       </c>
       <c r="S3" s="1">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="W3" s="1">
         <v>0</v>
       </c>
       <c r="X3" s="1">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="Y3" s="1" t="s">
         <v>1</v>
@@ -1132,7 +1132,7 @@
         <v>1</v>
       </c>
       <c r="AE3" s="1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="AF3" s="1" t="s">
         <v>16</v>
@@ -1141,7 +1141,7 @@
         <v>0</v>
       </c>
       <c r="AH3" s="1">
-        <v>32</v>
+        <v>162</v>
       </c>
       <c r="AI3" s="1" t="s">
         <v>1</v>
@@ -1156,7 +1156,7 @@
         <v>0</v>
       </c>
       <c r="AM3" s="1">
-        <v>15</v>
+        <v>158</v>
       </c>
       <c r="AN3" s="1" t="s">
         <v>1</v>
@@ -1176,31 +1176,31 @@
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C4" s="1">
         <v>0</v>
       </c>
       <c r="D4" s="1">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H4" s="1">
         <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>2</v>
+        <v>143</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>1</v>
@@ -1221,31 +1221,31 @@
         <v>1</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="R4" s="1">
         <v>0</v>
       </c>
       <c r="S4" s="1">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="T4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="W4" s="1">
         <v>0</v>
       </c>
       <c r="X4" s="1">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="1" t="s">
         <v>1</v>
@@ -1266,7 +1266,7 @@
         <v>1</v>
       </c>
       <c r="AE4" s="1" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="AF4" s="1" t="s">
         <v>16</v>
@@ -1275,7 +1275,7 @@
         <v>0</v>
       </c>
       <c r="AH4" s="1">
-        <v>162</v>
+        <v>32</v>
       </c>
       <c r="AI4" s="1" t="s">
         <v>1</v>
@@ -1310,56 +1310,56 @@
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>37</v>
+        <v>120</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C5" s="1">
         <v>0</v>
       </c>
       <c r="D5" s="1">
-        <v>0</v>
+        <v>212</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>67</v>
+        <v>102</v>
       </c>
       <c r="G5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1">
+        <v>2</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="M5" s="1">
+        <v>0</v>
+      </c>
+      <c r="N5" s="1">
+        <v>9</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="H5" s="1">
-        <v>0</v>
-      </c>
-      <c r="I5" s="1">
-        <v>0</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="M5" s="1">
-        <v>0</v>
-      </c>
-      <c r="N5" s="1">
-        <v>0</v>
-      </c>
-      <c r="O5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="R5" s="1">
         <v>0</v>
       </c>
@@ -1370,16 +1370,16 @@
         <v>1</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="W5" s="1">
         <v>0</v>
       </c>
       <c r="X5" s="1">
-        <v>120</v>
+        <v>63</v>
       </c>
       <c r="Y5" s="1" t="s">
         <v>1</v>
@@ -1415,90 +1415,90 @@
         <v>1</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
       <c r="AK5" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="AL5" s="1">
         <v>0</v>
       </c>
       <c r="AM5" s="1">
-        <v>64</v>
+        <v>211</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>56</v>
+        <v>109</v>
       </c>
       <c r="AP5" s="1" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="AQ5" s="1">
         <v>0</v>
       </c>
       <c r="AR5" s="1">
-        <v>23</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1">
+        <v>54</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M6" s="1">
+        <v>0</v>
+      </c>
+      <c r="N6" s="1">
+        <v>0</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1">
-        <v>0</v>
-      </c>
-      <c r="D6" s="1">
-        <v>0</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6" s="1">
-        <v>0</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M6" s="1">
-        <v>0</v>
-      </c>
-      <c r="N6" s="1">
-        <v>0</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="R6" s="1">
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="T6" s="1" t="s">
         <v>1</v>
@@ -1519,16 +1519,16 @@
         <v>1</v>
       </c>
       <c r="Z6" s="1" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="AA6" s="1" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="AB6" s="1">
         <v>0</v>
       </c>
       <c r="AC6" s="1">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="AD6" s="1" t="s">
         <v>1</v>
@@ -1549,16 +1549,16 @@
         <v>1</v>
       </c>
       <c r="AJ6" s="1" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="AK6" s="1" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="AL6" s="1">
         <v>0</v>
       </c>
       <c r="AM6" s="1">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="AN6" s="1" t="s">
         <v>1</v>
@@ -1578,10 +1578,10 @@
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>84</v>
+        <v>37</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="C7" s="1">
         <v>0</v>
@@ -1593,7 +1593,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>41</v>
@@ -1602,97 +1602,97 @@
         <v>0</v>
       </c>
       <c r="I7" s="1">
+        <v>145</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M7" s="1">
+        <v>0</v>
+      </c>
+      <c r="N7" s="1">
+        <v>0</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="R7" s="1">
+        <v>0</v>
+      </c>
+      <c r="S7" s="1">
+        <v>0</v>
+      </c>
+      <c r="T7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="V7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="W7" s="1">
+        <v>0</v>
+      </c>
+      <c r="X7" s="1">
+        <v>17</v>
+      </c>
+      <c r="Y7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="AA7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB7" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="1">
+        <v>36</v>
+      </c>
+      <c r="AD7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE7" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="AF7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG7" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH7" s="1">
+        <v>72</v>
+      </c>
+      <c r="AI7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AJ7" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="L7" s="1" t="s">
+      <c r="AK7" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="M7" s="1">
-        <v>0</v>
-      </c>
-      <c r="N7" s="1">
-        <v>69</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="R7" s="1">
-        <v>0</v>
-      </c>
-      <c r="S7" s="1">
-        <v>34</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="W7" s="1">
-        <v>0</v>
-      </c>
-      <c r="X7" s="1">
-        <v>72</v>
-      </c>
-      <c r="Y7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="Z7" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="AA7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="AB7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC7" s="1">
-        <v>23</v>
-      </c>
-      <c r="AD7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AE7" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="AF7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AG7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH7" s="1">
-        <v>130</v>
-      </c>
-      <c r="AI7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="AJ7" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="AK7" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="AL7" s="1">
         <v>0</v>
       </c>
       <c r="AM7" s="1">
-        <v>98</v>
+        <v>16</v>
       </c>
       <c r="AN7" s="1" t="s">
         <v>1</v>
@@ -1712,37 +1712,37 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="1">
-        <v>0</v>
-      </c>
-      <c r="D8" s="1">
-        <v>0</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="H8" s="1">
         <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>145</v>
+        <v>25</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="L8" s="1" t="s">
         <v>55</v>
@@ -1751,102 +1751,102 @@
         <v>0</v>
       </c>
       <c r="N8" s="1">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>29</v>
+        <v>113</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="R8" s="1">
         <v>0</v>
       </c>
       <c r="S8" s="1">
-        <v>89</v>
+        <v>10</v>
       </c>
       <c r="T8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="W8" s="1">
         <v>0</v>
       </c>
       <c r="X8" s="1">
-        <v>167</v>
+        <v>72</v>
       </c>
       <c r="Y8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="Z8" s="1" t="s">
-        <v>21</v>
+        <v>106</v>
       </c>
       <c r="AA8" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="AB8" s="1">
         <v>0</v>
       </c>
       <c r="AC8" s="1">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="AD8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AE8" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="AF8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AG8" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH8" s="1">
         <v>44</v>
       </c>
-      <c r="AF8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="AG8" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH8" s="1">
-        <v>58</v>
-      </c>
       <c r="AI8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AJ8" s="1" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="AK8" s="1" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="AL8" s="1">
         <v>0</v>
       </c>
       <c r="AM8" s="1">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="AN8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="AP8" s="1" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="AQ8" s="1">
         <v>0</v>
       </c>
       <c r="AR8" s="1">
-        <v>17</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>25</v>
@@ -1855,37 +1855,37 @@
         <v>0</v>
       </c>
       <c r="D9" s="1">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>27</v>
+        <v>67</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="H9" s="1">
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="M9" s="1">
         <v>0</v>
       </c>
       <c r="N9" s="1">
-        <v>9</v>
+        <v>98</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>1</v>
@@ -1906,16 +1906,16 @@
         <v>1</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="W9" s="1">
         <v>0</v>
       </c>
       <c r="X9" s="1">
-        <v>17</v>
+        <v>152</v>
       </c>
       <c r="Y9" s="1" t="s">
         <v>1</v>
@@ -1936,25 +1936,25 @@
         <v>1</v>
       </c>
       <c r="AE9" s="1" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="AF9" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="AG9" s="1">
         <v>0</v>
       </c>
       <c r="AH9" s="1">
-        <v>72</v>
+        <v>130</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AJ9" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="AK9" s="1" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="AL9" s="1">
         <v>0</v>
@@ -1966,60 +1966,60 @@
         <v>1</v>
       </c>
       <c r="AO9" s="1" t="s">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="AP9" s="1" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="AQ9" s="1">
         <v>0</v>
       </c>
       <c r="AR9" s="1">
-        <v>80</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="1">
+        <v>0</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="1">
-        <v>0</v>
-      </c>
-      <c r="D10" s="1">
-        <v>0</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="H10" s="1">
         <v>0</v>
       </c>
       <c r="I10" s="1">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="M10" s="1">
         <v>0</v>
       </c>
       <c r="N10" s="1">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>1</v>
@@ -2040,16 +2040,16 @@
         <v>1</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>87</v>
+        <v>20</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="W10" s="1">
         <v>0</v>
       </c>
       <c r="X10" s="1">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="Y10" s="1" t="s">
         <v>1</v>
@@ -2070,22 +2070,22 @@
         <v>1</v>
       </c>
       <c r="AE10" s="1" t="s">
-        <v>98</v>
+        <v>44</v>
       </c>
       <c r="AF10" s="1" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="AG10" s="1">
         <v>0</v>
       </c>
       <c r="AH10" s="1">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="AI10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="AJ10" s="1" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="AK10" s="1" t="s">
         <v>18</v>
@@ -2114,46 +2114,46 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>57</v>
+        <v>110</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C11" s="1">
         <v>0</v>
       </c>
       <c r="D11" s="1">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="H11" s="1">
         <v>0</v>
       </c>
       <c r="I11" s="1">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>68</v>
+        <v>103</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="M11" s="1">
         <v>0</v>
       </c>
       <c r="N11" s="1">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>1</v>
@@ -2174,7 +2174,7 @@
         <v>1</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="V11" s="1" t="s">
         <v>16</v>
@@ -2183,7 +2183,7 @@
         <v>0</v>
       </c>
       <c r="X11" s="1">
-        <v>84</v>
+        <v>167</v>
       </c>
       <c r="Y11" s="1" t="s">
         <v>1</v>
@@ -2263,16 +2263,16 @@
         <v>1</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="H12" s="1">
         <v>0</v>
       </c>
       <c r="I12" s="1">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>1</v>
@@ -2308,16 +2308,16 @@
         <v>1</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="W12" s="1">
         <v>0</v>
       </c>
       <c r="X12" s="1">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="Y12" s="1" t="s">
         <v>1</v>
@@ -2353,16 +2353,16 @@
         <v>1</v>
       </c>
       <c r="AJ12" s="1" t="s">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="AK12" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="AL12" s="1">
         <v>0</v>
       </c>
       <c r="AM12" s="1">
-        <v>89</v>
+        <v>0</v>
       </c>
       <c r="AN12" s="1" t="s">
         <v>1</v>
@@ -2382,31 +2382,31 @@
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>66</v>
+        <v>101</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C13" s="1">
         <v>0</v>
       </c>
       <c r="D13" s="1">
+        <v>12</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="G13" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H13" s="1">
         <v>0</v>
       </c>
       <c r="I13" s="1">
-        <v>125</v>
+        <v>86</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>1</v>
@@ -2442,16 +2442,16 @@
         <v>1</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="W13" s="1">
         <v>0</v>
       </c>
       <c r="X13" s="1">
-        <v>8</v>
+        <v>120</v>
       </c>
       <c r="Y13" s="1" t="s">
         <v>1</v>
@@ -2487,16 +2487,16 @@
         <v>1</v>
       </c>
       <c r="AJ13" s="1" t="s">
-        <v>73</v>
+        <v>123</v>
       </c>
       <c r="AK13" s="1" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="AL13" s="1">
         <v>0</v>
       </c>
       <c r="AM13" s="1">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="AN13" s="1" t="s">
         <v>1</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="1">
-        <v>344</v>
+        <v>418</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>1</v>
@@ -2540,7 +2540,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="1">
-        <v>517</v>
+        <v>535</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>378</v>
+        <v>466</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>1</v>
@@ -2570,7 +2570,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="1">
-        <v>282</v>
+        <v>354</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>1</v>
@@ -2585,7 +2585,7 @@
         <v>0</v>
       </c>
       <c r="X14" s="1">
-        <v>644</v>
+        <v>767</v>
       </c>
       <c r="Y14" s="1" t="s">
         <v>1</v>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="AC14" s="1">
-        <v>342</v>
+        <v>446</v>
       </c>
       <c r="AD14" s="1" t="s">
         <v>1</v>
@@ -2630,7 +2630,7 @@
         <v>0</v>
       </c>
       <c r="AM14" s="1">
-        <v>532</v>
+        <v>781</v>
       </c>
       <c r="AN14" s="1" t="s">
         <v>1</v>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>375</v>
+        <v>481</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 13
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FCDDA57-FBC0-48CD-B6EE-FA8CC9841D0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8805665B-69BC-44A8-B96E-C02CF1CCD869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
@@ -1042,16 +1042,16 @@
     </row>
     <row r="3" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C3" s="1">
         <v>0</v>
       </c>
       <c r="D3" s="1">
-        <v>52</v>
+        <v>278</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>123</v>
@@ -1096,7 +1096,7 @@
         <v>0</v>
       </c>
       <c r="S3" s="1">
-        <v>219</v>
+        <v>241</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>123</v>
@@ -1132,7 +1132,7 @@
         <v>123</v>
       </c>
       <c r="AE3" s="1" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="AF3" s="1" t="s">
         <v>15</v>
@@ -1141,7 +1141,7 @@
         <v>0</v>
       </c>
       <c r="AH3" s="1">
-        <v>121</v>
+        <v>242</v>
       </c>
       <c r="AI3" s="1" t="s">
         <v>123</v>
@@ -1176,16 +1176,16 @@
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C4" s="1">
         <v>0</v>
       </c>
       <c r="D4" s="1">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>123</v>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>123</v>
@@ -1221,16 +1221,16 @@
         <v>123</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="R4" s="1">
         <v>0</v>
       </c>
       <c r="S4" s="1">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="T4" s="1" t="s">
         <v>123</v>
@@ -1260,22 +1260,22 @@
         <v>0</v>
       </c>
       <c r="AC4" s="1">
-        <v>82</v>
+        <v>130</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE4" s="1" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="AF4" s="1" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="AG4" s="1">
         <v>0</v>
       </c>
       <c r="AH4" s="1">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="AI4" s="1" t="s">
         <v>123</v>
@@ -1310,10 +1310,10 @@
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1">
         <v>0</v>
@@ -1355,10 +1355,10 @@
         <v>123</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="R5" s="1">
         <v>0</v>
@@ -1400,7 +1400,7 @@
         <v>123</v>
       </c>
       <c r="AE5" s="1" t="s">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="AF5" s="1" t="s">
         <v>15</v>
@@ -1409,7 +1409,7 @@
         <v>0</v>
       </c>
       <c r="AH5" s="1">
-        <v>0</v>
+        <v>137</v>
       </c>
       <c r="AI5" s="1" t="s">
         <v>123</v>
@@ -1444,16 +1444,16 @@
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="C6" s="1">
         <v>0</v>
       </c>
       <c r="D6" s="1">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>123</v>
@@ -1489,16 +1489,16 @@
         <v>123</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="R6" s="1">
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="T6" s="1" t="s">
         <v>123</v>
@@ -1534,16 +1534,16 @@
         <v>123</v>
       </c>
       <c r="AE6" s="1" t="s">
-        <v>106</v>
+        <v>52</v>
       </c>
       <c r="AF6" s="1" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="AG6" s="1">
         <v>0</v>
       </c>
       <c r="AH6" s="1">
-        <v>224</v>
+        <v>0</v>
       </c>
       <c r="AI6" s="1" t="s">
         <v>123</v>
@@ -1578,16 +1578,16 @@
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0</v>
+      </c>
+      <c r="D7" s="1">
         <v>24</v>
-      </c>
-      <c r="C7" s="1">
-        <v>0</v>
-      </c>
-      <c r="D7" s="1">
-        <v>0</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>123</v>
@@ -1617,22 +1617,22 @@
         <v>0</v>
       </c>
       <c r="N7" s="1">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="R7" s="1">
         <v>0</v>
       </c>
       <c r="S7" s="1">
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="T7" s="1" t="s">
         <v>123</v>
@@ -1668,16 +1668,16 @@
         <v>123</v>
       </c>
       <c r="AE7" s="1" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="AF7" s="1" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="AG7" s="1">
         <v>0</v>
       </c>
       <c r="AH7" s="1">
-        <v>177</v>
+        <v>0</v>
       </c>
       <c r="AI7" s="1" t="s">
         <v>123</v>
@@ -1692,7 +1692,7 @@
         <v>0</v>
       </c>
       <c r="AM7" s="1">
-        <v>185</v>
+        <v>358</v>
       </c>
       <c r="AN7" s="1" t="s">
         <v>123</v>
@@ -1712,10 +1712,10 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C8" s="1">
         <v>0</v>
@@ -1757,16 +1757,16 @@
         <v>123</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>112</v>
+        <v>68</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="R8" s="1">
         <v>0</v>
       </c>
       <c r="S8" s="1">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="T8" s="1" t="s">
         <v>123</v>
@@ -1802,16 +1802,16 @@
         <v>123</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>22</v>
+        <v>106</v>
       </c>
       <c r="AF8" s="1" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="AG8" s="1">
         <v>0</v>
       </c>
       <c r="AH8" s="1">
-        <v>233</v>
+        <v>294</v>
       </c>
       <c r="AI8" s="1" t="s">
         <v>123</v>
@@ -1846,10 +1846,10 @@
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9" s="1">
         <v>0</v>
@@ -1891,16 +1891,16 @@
         <v>123</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>28</v>
+        <v>112</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="R9" s="1">
         <v>0</v>
       </c>
       <c r="S9" s="1">
-        <v>161</v>
+        <v>34</v>
       </c>
       <c r="T9" s="1" t="s">
         <v>123</v>
@@ -1915,7 +1915,7 @@
         <v>0</v>
       </c>
       <c r="X9" s="1">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="Y9" s="1" t="s">
         <v>123</v>
@@ -1936,16 +1936,16 @@
         <v>123</v>
       </c>
       <c r="AE9" s="1" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AF9" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AG9" s="1">
         <v>0</v>
       </c>
       <c r="AH9" s="1">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>123</v>
@@ -1980,16 +1980,16 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C10" s="1">
         <v>0</v>
       </c>
       <c r="D10" s="1">
-        <v>239</v>
+        <v>0</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>123</v>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
       <c r="I10" s="1">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>123</v>
@@ -2025,16 +2025,16 @@
         <v>123</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="R10" s="1">
         <v>0</v>
       </c>
       <c r="S10" s="1">
-        <v>58</v>
+        <v>161</v>
       </c>
       <c r="T10" s="1" t="s">
         <v>123</v>
@@ -2049,7 +2049,7 @@
         <v>0</v>
       </c>
       <c r="X10" s="1">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="Y10" s="1" t="s">
         <v>123</v>
@@ -2070,16 +2070,16 @@
         <v>123</v>
       </c>
       <c r="AE10" s="1" t="s">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="AF10" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="AG10" s="1">
         <v>0</v>
       </c>
       <c r="AH10" s="1">
-        <v>155</v>
+        <v>188</v>
       </c>
       <c r="AI10" s="1" t="s">
         <v>123</v>
@@ -2114,16 +2114,16 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>46</v>
+        <v>119</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="C11" s="1">
         <v>0</v>
       </c>
       <c r="D11" s="1">
-        <v>189</v>
+        <v>239</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>123</v>
@@ -2204,16 +2204,16 @@
         <v>123</v>
       </c>
       <c r="AE11" s="1" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="AF11" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="AG11" s="1">
         <v>0</v>
       </c>
       <c r="AH11" s="1">
-        <v>25</v>
+        <v>213</v>
       </c>
       <c r="AI11" s="1" t="s">
         <v>123</v>
@@ -2338,16 +2338,16 @@
         <v>123</v>
       </c>
       <c r="AE12" s="1" t="s">
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="AF12" s="1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="AG12" s="1">
         <v>0</v>
       </c>
       <c r="AH12" s="1">
-        <v>68</v>
+        <v>25</v>
       </c>
       <c r="AI12" s="1" t="s">
         <v>123</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="1">
-        <v>573</v>
+        <v>662</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>123</v>
@@ -2540,7 +2540,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="1">
-        <v>1077</v>
+        <v>1100</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>123</v>
@@ -2555,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>123</v>
@@ -2570,7 +2570,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="1">
-        <v>868</v>
+        <v>972</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>123</v>
@@ -2585,7 +2585,7 @@
         <v>0</v>
       </c>
       <c r="X14" s="1">
-        <v>1171</v>
+        <v>1216</v>
       </c>
       <c r="Y14" s="1" t="s">
         <v>123</v>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="AC14" s="1">
-        <v>932</v>
+        <v>980</v>
       </c>
       <c r="AD14" s="1" t="s">
         <v>123</v>
@@ -2615,7 +2615,7 @@
         <v>0</v>
       </c>
       <c r="AH14" s="1">
-        <v>1259</v>
+        <v>1456</v>
       </c>
       <c r="AI14" s="1" t="s">
         <v>123</v>
@@ -2630,7 +2630,7 @@
         <v>0</v>
       </c>
       <c r="AM14" s="1">
-        <v>1354</v>
+        <v>1527</v>
       </c>
       <c r="AN14" s="1" t="s">
         <v>123</v>

</xml_diff>